<commit_message>
v3.0: feat - CTQ
</commit_message>
<xml_diff>
--- a/resources/M626/spc_sheet_oos_detail.xlsx
+++ b/resources/M626/spc_sheet_oos_detail.xlsx
@@ -2001,7 +2001,7 @@
         <v>-6.5497</v>
       </c>
       <c r="I15">
-        <v>0.4878552631578948</v>
+        <v>0.4878552631578947</v>
       </c>
       <c r="J15">
         <v>6.5</v>
@@ -2077,7 +2077,7 @@
         <v>-6.853</v>
       </c>
       <c r="I17">
-        <v>-0.05989736842105262</v>
+        <v>-0.05989736842105266</v>
       </c>
       <c r="J17">
         <v>6.5</v>
@@ -2191,7 +2191,7 @@
         <v>-6.5725</v>
       </c>
       <c r="I20">
-        <v>0.3449543859649122</v>
+        <v>0.3449543859649123</v>
       </c>
       <c r="J20">
         <v>6.5</v>
@@ -2229,7 +2229,7 @@
         <v>-5.9993</v>
       </c>
       <c r="I21">
-        <v>0.717057894736842</v>
+        <v>0.7170578947368421</v>
       </c>
       <c r="J21">
         <v>6.5</v>
@@ -2533,7 +2533,7 @@
         <v>-7.5177</v>
       </c>
       <c r="I29">
-        <v>-0.8770456140350879</v>
+        <v>-0.8770456140350877</v>
       </c>
       <c r="J29">
         <v>6.5</v>
@@ -2609,7 +2609,7 @@
         <v>-6.5326</v>
       </c>
       <c r="I31">
-        <v>0.007044736842105248</v>
+        <v>0.007044736842105261</v>
       </c>
       <c r="J31">
         <v>6.5</v>
@@ -2647,7 +2647,7 @@
         <v>-8.8163</v>
       </c>
       <c r="I32">
-        <v>0.04442543859649123</v>
+        <v>0.04442543859649125</v>
       </c>
       <c r="J32">
         <v>6.5</v>
@@ -2913,7 +2913,7 @@
         <v>-8.9923</v>
       </c>
       <c r="I39">
-        <v>-0.3703271929824561</v>
+        <v>-0.3703271929824562</v>
       </c>
       <c r="J39">
         <v>6.5</v>
@@ -3939,7 +3939,7 @@
         <v>-6.9495</v>
       </c>
       <c r="I66">
-        <v>0.09059122807017543</v>
+        <v>0.09059122807017542</v>
       </c>
       <c r="J66">
         <v>6.5</v>
@@ -4129,7 +4129,7 @@
         <v>-7.3274</v>
       </c>
       <c r="I71">
-        <v>0.02795575221238938</v>
+        <v>0.02795575221238936</v>
       </c>
       <c r="J71">
         <v>6.5</v>
@@ -4889,7 +4889,7 @@
         <v>-5.1754</v>
       </c>
       <c r="I91">
-        <v>-0.3718087719298245</v>
+        <v>-0.3718087719298246</v>
       </c>
       <c r="J91">
         <v>6.5</v>
@@ -5573,7 +5573,7 @@
         <v>-5.9765</v>
       </c>
       <c r="I109">
-        <v>0.2397718181818182</v>
+        <v>0.2397718181818181</v>
       </c>
       <c r="J109">
         <v>6.5</v>
@@ -5839,7 +5839,7 @@
         <v>-6.7429</v>
       </c>
       <c r="I116">
-        <v>-0.8630114035087718</v>
+        <v>-0.8630114035087719</v>
       </c>
       <c r="J116">
         <v>6.5</v>
@@ -7321,7 +7321,7 @@
         <v>-6.7592</v>
       </c>
       <c r="I155">
-        <v>0.2844389380530973</v>
+        <v>0.2844389380530974</v>
       </c>
       <c r="J155">
         <v>6.5</v>
@@ -7435,7 +7435,7 @@
         <v>-8.3222</v>
       </c>
       <c r="I158">
-        <v>-0.3694438596491229</v>
+        <v>-0.3694438596491228</v>
       </c>
       <c r="J158">
         <v>6.5</v>
@@ -7473,7 +7473,7 @@
         <v>-7.1162</v>
       </c>
       <c r="I159">
-        <v>0.02907345132743362</v>
+        <v>0.02907345132743365</v>
       </c>
       <c r="J159">
         <v>6.5</v>
@@ -8081,7 +8081,7 @@
         <v>-7.0164</v>
       </c>
       <c r="I175">
-        <v>0.05691666666666671</v>
+        <v>0.05691666666666669</v>
       </c>
       <c r="J175">
         <v>6.5</v>
@@ -8157,7 +8157,7 @@
         <v>-6.5805</v>
       </c>
       <c r="I177">
-        <v>-0.5253763157894736</v>
+        <v>-0.5253763157894737</v>
       </c>
       <c r="J177">
         <v>6.5</v>
@@ -8537,7 +8537,7 @@
         <v>-4.7025</v>
       </c>
       <c r="I187">
-        <v>0.1291447368421053</v>
+        <v>0.1291447368421052</v>
       </c>
       <c r="J187">
         <v>6.5</v>
@@ -8613,7 +8613,7 @@
         <v>-6.7699</v>
       </c>
       <c r="I189">
-        <v>-0.3602491228070175</v>
+        <v>-0.3602491228070176</v>
       </c>
       <c r="J189">
         <v>6.5</v>
@@ -8917,7 +8917,7 @@
         <v>-6.6607</v>
       </c>
       <c r="I197">
-        <v>0.438721052631579</v>
+        <v>0.4387210526315789</v>
       </c>
       <c r="J197">
         <v>6.5</v>
@@ -9411,7 +9411,7 @@
         <v>-6.5279</v>
       </c>
       <c r="I210">
-        <v>-0.3397394736842105</v>
+        <v>-0.3397394736842106</v>
       </c>
       <c r="J210">
         <v>6.5</v>
@@ -9753,7 +9753,7 @@
         <v>-7.2139</v>
       </c>
       <c r="I219">
-        <v>0.8870140350877193</v>
+        <v>0.8870140350877194</v>
       </c>
       <c r="J219">
         <v>6.5</v>
@@ -9905,7 +9905,7 @@
         <v>-5.6397</v>
       </c>
       <c r="I223">
-        <v>0.4995482456140351</v>
+        <v>0.499548245614035</v>
       </c>
       <c r="J223">
         <v>6.5</v>
@@ -10589,7 +10589,7 @@
         <v>-5.2818</v>
       </c>
       <c r="I241">
-        <v>-0.5151245614035087</v>
+        <v>-0.5151245614035088</v>
       </c>
       <c r="J241">
         <v>6.5</v>
@@ -10779,7 +10779,7 @@
         <v>-5.1609</v>
       </c>
       <c r="I246">
-        <v>-0.03773245614035088</v>
+        <v>-0.03773245614035086</v>
       </c>
       <c r="J246">
         <v>6.5</v>
@@ -10817,7 +10817,7 @@
         <v>-7.5475</v>
       </c>
       <c r="I247">
-        <v>0.00142631578947371</v>
+        <v>0.001426315789473696</v>
       </c>
       <c r="J247">
         <v>6.5</v>
@@ -10893,7 +10893,7 @@
         <v>-5.224</v>
       </c>
       <c r="I249">
-        <v>0.5808824561403509</v>
+        <v>0.5808824561403508</v>
       </c>
       <c r="J249">
         <v>6.5</v>
@@ -11121,7 +11121,7 @@
         <v>-4.9299</v>
       </c>
       <c r="I255">
-        <v>-0.08569999999999998</v>
+        <v>-0.0857</v>
       </c>
       <c r="J255">
         <v>6.5</v>
@@ -11197,7 +11197,7 @@
         <v>-4.7771</v>
       </c>
       <c r="I257">
-        <v>-0.3050263157894737</v>
+        <v>-0.3050263157894736</v>
       </c>
       <c r="J257">
         <v>6.5</v>
@@ -11995,7 +11995,7 @@
         <v>-9.602600000000001</v>
       </c>
       <c r="I278">
-        <v>-0.3922938053097345</v>
+        <v>-0.3922938053097346</v>
       </c>
       <c r="J278">
         <v>6.5</v>
@@ -12109,7 +12109,7 @@
         <v>-7.4181</v>
       </c>
       <c r="I281">
-        <v>-0.8477921052631578</v>
+        <v>-0.847792105263158</v>
       </c>
       <c r="J281">
         <v>6.5</v>
@@ -12261,7 +12261,7 @@
         <v>-4.3077</v>
       </c>
       <c r="I285">
-        <v>0.003302631578947369</v>
+        <v>0.003302631578947381</v>
       </c>
       <c r="J285">
         <v>6.5</v>
@@ -12907,7 +12907,7 @@
         <v>-5.7208</v>
       </c>
       <c r="I302">
-        <v>-0.869777192982456</v>
+        <v>-0.8697771929824561</v>
       </c>
       <c r="J302">
         <v>6.5</v>
@@ -13363,7 +13363,7 @@
         <v>-2.644</v>
       </c>
       <c r="I314">
-        <v>1.357429824561403</v>
+        <v>1.357429824561404</v>
       </c>
       <c r="J314">
         <v>6.5</v>
@@ -13781,7 +13781,7 @@
         <v>-3.2937</v>
       </c>
       <c r="I325">
-        <v>0.6668903508771931</v>
+        <v>0.666890350877193</v>
       </c>
       <c r="J325">
         <v>6.5</v>
@@ -13857,7 +13857,7 @@
         <v>-5.6367</v>
       </c>
       <c r="I327">
-        <v>0.489328947368421</v>
+        <v>0.4893289473684211</v>
       </c>
       <c r="J327">
         <v>6.5</v>
@@ -13933,7 +13933,7 @@
         <v>-5.9722</v>
       </c>
       <c r="I329">
-        <v>-0.09155877192982456</v>
+        <v>-0.09155877192982455</v>
       </c>
       <c r="J329">
         <v>6.5</v>
@@ -14161,7 +14161,7 @@
         <v>-7.0553</v>
       </c>
       <c r="I335">
-        <v>-0.9032403508771929</v>
+        <v>-0.903240350877193</v>
       </c>
       <c r="J335">
         <v>6.5</v>
@@ -15339,7 +15339,7 @@
         <v>-6.6445</v>
       </c>
       <c r="I366">
-        <v>0.03264736842105264</v>
+        <v>0.03264736842105263</v>
       </c>
       <c r="J366">
         <v>6.5</v>
@@ -16023,7 +16023,7 @@
         <v>-6.6968</v>
       </c>
       <c r="I384">
-        <v>-0.2789184210526315</v>
+        <v>-0.2789184210526316</v>
       </c>
       <c r="J384">
         <v>6.5</v>
@@ -16175,7 +16175,7 @@
         <v>-8.2082</v>
       </c>
       <c r="I388">
-        <v>0.08817894736842105</v>
+        <v>0.08817894736842108</v>
       </c>
       <c r="J388">
         <v>6.5</v>
@@ -18075,7 +18075,7 @@
         <v>-6.0461</v>
       </c>
       <c r="I438">
-        <v>0.6397596491228071</v>
+        <v>0.6397596491228069</v>
       </c>
       <c r="J438">
         <v>6.5</v>
@@ -19899,7 +19899,7 @@
         <v>-6.237</v>
       </c>
       <c r="I486">
-        <v>0.1851447368421053</v>
+        <v>0.1851447368421052</v>
       </c>
       <c r="J486">
         <v>6.5</v>
@@ -20279,7 +20279,7 @@
         <v>-6.1561</v>
       </c>
       <c r="I496">
-        <v>-0.08215350877192983</v>
+        <v>-0.08215350877192981</v>
       </c>
       <c r="J496">
         <v>6.5</v>
@@ -20735,7 +20735,7 @@
         <v>-5.9368</v>
       </c>
       <c r="I508">
-        <v>-0.004456140350877168</v>
+        <v>-0.004456140350877196</v>
       </c>
       <c r="J508">
         <v>6.5</v>
@@ -21761,7 +21761,7 @@
         <v>-5.2677</v>
       </c>
       <c r="I535">
-        <v>0.5644705357142857</v>
+        <v>0.5644705357142856</v>
       </c>
       <c r="J535">
         <v>6.5</v>
@@ -21799,7 +21799,7 @@
         <v>-4.8043</v>
       </c>
       <c r="I536">
-        <v>0.3505271929824562</v>
+        <v>0.3505271929824561</v>
       </c>
       <c r="J536">
         <v>6.5</v>
@@ -22027,7 +22027,7 @@
         <v>-10.0195</v>
       </c>
       <c r="I542">
-        <v>0.03782368421052631</v>
+        <v>0.03782368421052629</v>
       </c>
       <c r="J542">
         <v>6.5</v>
@@ -22977,7 +22977,7 @@
         <v>-6.8548</v>
       </c>
       <c r="I567">
-        <v>-0.489969298245614</v>
+        <v>-0.4899692982456141</v>
       </c>
       <c r="J567">
         <v>6.5</v>
@@ -23281,7 +23281,7 @@
         <v>-6.7318</v>
       </c>
       <c r="I575">
-        <v>0.09459649122807018</v>
+        <v>0.09459649122807019</v>
       </c>
       <c r="J575">
         <v>6.5</v>
@@ -23395,7 +23395,7 @@
         <v>-4.8922</v>
       </c>
       <c r="I578">
-        <v>-0.7553938596491228</v>
+        <v>-0.7553938596491229</v>
       </c>
       <c r="J578">
         <v>6.5</v>
@@ -23775,7 +23775,7 @@
         <v>-7.9624</v>
       </c>
       <c r="I588">
-        <v>-0.1399333333333334</v>
+        <v>-0.1399333333333333</v>
       </c>
       <c r="J588">
         <v>6.5</v>
@@ -24117,7 +24117,7 @@
         <v>-3.8887</v>
       </c>
       <c r="I597">
-        <v>-0.09209473684210527</v>
+        <v>-0.09209473684210528</v>
       </c>
       <c r="J597">
         <v>6.5</v>
@@ -24459,7 +24459,7 @@
         <v>-6.0164</v>
       </c>
       <c r="I606">
-        <v>0.7425824561403508</v>
+        <v>0.742582456140351</v>
       </c>
       <c r="J606">
         <v>6.5</v>
@@ -25485,7 +25485,7 @@
         <v>-4.5379</v>
       </c>
       <c r="I633">
-        <v>0.8886482456140352</v>
+        <v>0.888648245614035</v>
       </c>
       <c r="J633">
         <v>6.5</v>
@@ -25561,7 +25561,7 @@
         <v>-6.8984</v>
       </c>
       <c r="I635">
-        <v>-2.148637719298246</v>
+        <v>-2.148637719298245</v>
       </c>
       <c r="J635">
         <v>6.5</v>
@@ -25599,7 +25599,7 @@
         <v>-1.9388</v>
       </c>
       <c r="I636">
-        <v>2.021550877192983</v>
+        <v>2.021550877192982</v>
       </c>
       <c r="J636">
         <v>6.5</v>

</xml_diff>

<commit_message>
v3.1: feat - rendering sync
</commit_message>
<xml_diff>
--- a/resources/M626/spc_sheet_oos_detail.xlsx
+++ b/resources/M626/spc_sheet_oos_detail.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="41">
   <si>
     <t>factory</t>
   </si>
@@ -50,12 +50,102 @@
   </si>
   <si>
     <t>oos_type</t>
+  </si>
+  <si>
+    <t>OLED</t>
+  </si>
+  <si>
+    <t>M626</t>
+  </si>
+  <si>
+    <t>21200</t>
+  </si>
+  <si>
+    <t>PPA_B_X</t>
+  </si>
+  <si>
+    <t>PPA_B_Y</t>
+  </si>
+  <si>
+    <t>PPA_G1_X</t>
+  </si>
+  <si>
+    <t>PPA_G1_Y</t>
+  </si>
+  <si>
+    <t>PPA_G_Y</t>
+  </si>
+  <si>
+    <t>PPA_R1_Y</t>
+  </si>
+  <si>
+    <t>PPA_R_X</t>
+  </si>
+  <si>
+    <t>PPA_R_Y</t>
+  </si>
+  <si>
+    <t>L3MY6501S252</t>
+  </si>
+  <si>
+    <t>L3MY6501U161</t>
+  </si>
+  <si>
+    <t>L3MY6501U052</t>
+  </si>
+  <si>
+    <t>L3MY6501Q031</t>
+  </si>
+  <si>
+    <t>L3MY6501R022</t>
+  </si>
+  <si>
+    <t>L3MY6501S201</t>
+  </si>
+  <si>
+    <t>L3MY6501T161</t>
+  </si>
+  <si>
+    <t>L3MY6501N271</t>
+  </si>
+  <si>
+    <t>L3MY6501P121</t>
+  </si>
+  <si>
+    <t>L3MY6501P022</t>
+  </si>
+  <si>
+    <t>L3MY6501Q222</t>
+  </si>
+  <si>
+    <t>L3MY6501U121</t>
+  </si>
+  <si>
+    <t>L3MY6501R121</t>
+  </si>
+  <si>
+    <t>L3MY6501R161</t>
+  </si>
+  <si>
+    <t>L3MY6501N172</t>
+  </si>
+  <si>
+    <t>LSL</t>
+  </si>
+  <si>
+    <t>USL/LSL</t>
+  </si>
+  <si>
+    <t>USL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -108,11 +198,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -448,6 +539,1032 @@
         <v>11</v>
       </c>
     </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46205.47403935185</v>
+      </c>
+      <c r="G2">
+        <v>3.8436</v>
+      </c>
+      <c r="H2">
+        <v>-6.6488</v>
+      </c>
+      <c r="I2">
+        <v>-0.579058407079646</v>
+      </c>
+      <c r="J2">
+        <v>6.5</v>
+      </c>
+      <c r="K2">
+        <v>-6.5</v>
+      </c>
+      <c r="L2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46205.50491898148</v>
+      </c>
+      <c r="G3">
+        <v>6.8913</v>
+      </c>
+      <c r="H3">
+        <v>-6.8436</v>
+      </c>
+      <c r="I3">
+        <v>0.2694433628318584</v>
+      </c>
+      <c r="J3">
+        <v>6.5</v>
+      </c>
+      <c r="K3">
+        <v>-6.5</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46205.98925925926</v>
+      </c>
+      <c r="G4">
+        <v>7.3391</v>
+      </c>
+      <c r="H4">
+        <v>-5.4987</v>
+      </c>
+      <c r="I4">
+        <v>1.151083333333333</v>
+      </c>
+      <c r="J4">
+        <v>6.5</v>
+      </c>
+      <c r="K4">
+        <v>-6.5</v>
+      </c>
+      <c r="L4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46206.52177083334</v>
+      </c>
+      <c r="G5">
+        <v>7.4699</v>
+      </c>
+      <c r="H5">
+        <v>-7.3274</v>
+      </c>
+      <c r="I5">
+        <v>0.02795575221238938</v>
+      </c>
+      <c r="J5">
+        <v>6.5</v>
+      </c>
+      <c r="K5">
+        <v>-6.5</v>
+      </c>
+      <c r="L5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46204.30900462963</v>
+      </c>
+      <c r="G6">
+        <v>6.5551</v>
+      </c>
+      <c r="H6">
+        <v>-3.753</v>
+      </c>
+      <c r="I6">
+        <v>0.6958912280701753</v>
+      </c>
+      <c r="J6">
+        <v>6.5</v>
+      </c>
+      <c r="K6">
+        <v>-6.5</v>
+      </c>
+      <c r="L6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46204.8665625</v>
+      </c>
+      <c r="G7">
+        <v>4.7678</v>
+      </c>
+      <c r="H7">
+        <v>-7.4633</v>
+      </c>
+      <c r="I7">
+        <v>-1.287028571428571</v>
+      </c>
+      <c r="J7">
+        <v>6.5</v>
+      </c>
+      <c r="K7">
+        <v>-6.5</v>
+      </c>
+      <c r="L7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46205.50491898148</v>
+      </c>
+      <c r="G8">
+        <v>7.1197</v>
+      </c>
+      <c r="H8">
+        <v>-4.5</v>
+      </c>
+      <c r="I8">
+        <v>1.028345132743363</v>
+      </c>
+      <c r="J8">
+        <v>6.5</v>
+      </c>
+      <c r="K8">
+        <v>-6.5</v>
+      </c>
+      <c r="L8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46205.98925925926</v>
+      </c>
+      <c r="G9">
+        <v>4.1703</v>
+      </c>
+      <c r="H9">
+        <v>-6.7701</v>
+      </c>
+      <c r="I9">
+        <v>-0.5932921052631579</v>
+      </c>
+      <c r="J9">
+        <v>6.5</v>
+      </c>
+      <c r="K9">
+        <v>-6.5</v>
+      </c>
+      <c r="L9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46206.02383101852</v>
+      </c>
+      <c r="G10">
+        <v>5.8846</v>
+      </c>
+      <c r="H10">
+        <v>-7.298</v>
+      </c>
+      <c r="I10">
+        <v>-0.8348867256637169</v>
+      </c>
+      <c r="J10">
+        <v>6.5</v>
+      </c>
+      <c r="K10">
+        <v>-6.5</v>
+      </c>
+      <c r="L10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46206.45180555555</v>
+      </c>
+      <c r="G11">
+        <v>7.4676</v>
+      </c>
+      <c r="H11">
+        <v>-5.8927</v>
+      </c>
+      <c r="I11">
+        <v>0.1450061946902655</v>
+      </c>
+      <c r="J11">
+        <v>6.5</v>
+      </c>
+      <c r="K11">
+        <v>-6.5</v>
+      </c>
+      <c r="L11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="2">
+        <v>46206.52177083334</v>
+      </c>
+      <c r="G12">
+        <v>7.3647</v>
+      </c>
+      <c r="H12">
+        <v>-3.3418</v>
+      </c>
+      <c r="I12">
+        <v>2.13499203539823</v>
+      </c>
+      <c r="J12">
+        <v>6.5</v>
+      </c>
+      <c r="K12">
+        <v>-6.5</v>
+      </c>
+      <c r="L12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="2">
+        <v>46207.14076388889</v>
+      </c>
+      <c r="G13">
+        <v>6.52</v>
+      </c>
+      <c r="H13">
+        <v>-4.1674</v>
+      </c>
+      <c r="I13">
+        <v>0.03299017857142859</v>
+      </c>
+      <c r="J13">
+        <v>6.5</v>
+      </c>
+      <c r="K13">
+        <v>-6.5</v>
+      </c>
+      <c r="L13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46207.17734953704</v>
+      </c>
+      <c r="G14">
+        <v>5.5108</v>
+      </c>
+      <c r="H14">
+        <v>-7.0698</v>
+      </c>
+      <c r="I14">
+        <v>0.521209009009009</v>
+      </c>
+      <c r="J14">
+        <v>6.5</v>
+      </c>
+      <c r="K14">
+        <v>-6.5</v>
+      </c>
+      <c r="L14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="2">
+        <v>46205.98925925926</v>
+      </c>
+      <c r="G15">
+        <v>6.9491</v>
+      </c>
+      <c r="H15">
+        <v>-4.4926</v>
+      </c>
+      <c r="I15">
+        <v>0.8067271929824561</v>
+      </c>
+      <c r="J15">
+        <v>6.5</v>
+      </c>
+      <c r="K15">
+        <v>-6.5</v>
+      </c>
+      <c r="L15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16" s="2">
+        <v>46206.02383101852</v>
+      </c>
+      <c r="G16">
+        <v>7.648</v>
+      </c>
+      <c r="H16">
+        <v>-5.7208</v>
+      </c>
+      <c r="I16">
+        <v>-0.8697771929824561</v>
+      </c>
+      <c r="J16">
+        <v>6.5</v>
+      </c>
+      <c r="K16">
+        <v>-6.5</v>
+      </c>
+      <c r="L16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="2">
+        <v>46207.17734953704</v>
+      </c>
+      <c r="G17">
+        <v>6.1083</v>
+      </c>
+      <c r="H17">
+        <v>-6.5466</v>
+      </c>
+      <c r="I17">
+        <v>-0.7771561403508772</v>
+      </c>
+      <c r="J17">
+        <v>6.5</v>
+      </c>
+      <c r="K17">
+        <v>-6.5</v>
+      </c>
+      <c r="L17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" t="s">
+        <v>18</v>
+      </c>
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="2">
+        <v>46206.05597222222</v>
+      </c>
+      <c r="G18">
+        <v>7.429</v>
+      </c>
+      <c r="H18">
+        <v>-4.3552</v>
+      </c>
+      <c r="I18">
+        <v>1.858010526315789</v>
+      </c>
+      <c r="J18">
+        <v>6.5</v>
+      </c>
+      <c r="K18">
+        <v>-6.5</v>
+      </c>
+      <c r="L18" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="2">
+        <v>46207.17734953704</v>
+      </c>
+      <c r="G19">
+        <v>6.5012</v>
+      </c>
+      <c r="H19">
+        <v>-4.973</v>
+      </c>
+      <c r="I19">
+        <v>1.165839473684211</v>
+      </c>
+      <c r="J19">
+        <v>6.5</v>
+      </c>
+      <c r="K19">
+        <v>-6.5</v>
+      </c>
+      <c r="L19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="2">
+        <v>46205.98925925926</v>
+      </c>
+      <c r="G20">
+        <v>6.8508</v>
+      </c>
+      <c r="H20">
+        <v>-3.2823</v>
+      </c>
+      <c r="I20">
+        <v>1.517928947368421</v>
+      </c>
+      <c r="J20">
+        <v>6.5</v>
+      </c>
+      <c r="K20">
+        <v>-6.5</v>
+      </c>
+      <c r="L20" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21" s="2">
+        <v>46206.45180555555</v>
+      </c>
+      <c r="G21">
+        <v>6.6823</v>
+      </c>
+      <c r="H21">
+        <v>-6.5792</v>
+      </c>
+      <c r="I21">
+        <v>1.075626548672566</v>
+      </c>
+      <c r="J21">
+        <v>6.5</v>
+      </c>
+      <c r="K21">
+        <v>-6.5</v>
+      </c>
+      <c r="L21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="2">
+        <v>46206.52177083334</v>
+      </c>
+      <c r="G22">
+        <v>6.7933</v>
+      </c>
+      <c r="H22">
+        <v>-1.7444</v>
+      </c>
+      <c r="I22">
+        <v>2.203963716814159</v>
+      </c>
+      <c r="J22">
+        <v>6.5</v>
+      </c>
+      <c r="K22">
+        <v>-6.5</v>
+      </c>
+      <c r="L22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="2">
+        <v>46205.43644675926</v>
+      </c>
+      <c r="G23">
+        <v>6.5487</v>
+      </c>
+      <c r="H23">
+        <v>-3.0655</v>
+      </c>
+      <c r="I23">
+        <v>1.095975438596491</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23">
+        <v>-6.5</v>
+      </c>
+      <c r="L23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" s="2">
+        <v>46206.02383101852</v>
+      </c>
+      <c r="G24">
+        <v>6.815</v>
+      </c>
+      <c r="H24">
+        <v>-5.1156</v>
+      </c>
+      <c r="I24">
+        <v>0.8954052631578947</v>
+      </c>
+      <c r="J24">
+        <v>6.5</v>
+      </c>
+      <c r="K24">
+        <v>-6.5</v>
+      </c>
+      <c r="L24" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="2">
+        <v>46204.27109953704</v>
+      </c>
+      <c r="G25">
+        <v>7.2283</v>
+      </c>
+      <c r="H25">
+        <v>-3.8887</v>
+      </c>
+      <c r="I25">
+        <v>-0.09209473684210527</v>
+      </c>
+      <c r="J25">
+        <v>6.5</v>
+      </c>
+      <c r="K25">
+        <v>-6.5</v>
+      </c>
+      <c r="L25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" s="2">
+        <v>46204.35930555555</v>
+      </c>
+      <c r="G26">
+        <v>6.9917</v>
+      </c>
+      <c r="H26">
+        <v>-5.5588</v>
+      </c>
+      <c r="I26">
+        <v>-0.9715920353982301</v>
+      </c>
+      <c r="J26">
+        <v>6.5</v>
+      </c>
+      <c r="K26">
+        <v>-6.5</v>
+      </c>
+      <c r="L26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27" s="2">
+        <v>46206.45180555555</v>
+      </c>
+      <c r="G27">
+        <v>7.5327</v>
+      </c>
+      <c r="H27">
+        <v>-9.287100000000001</v>
+      </c>
+      <c r="I27">
+        <v>-0.3583557522123894</v>
+      </c>
+      <c r="J27">
+        <v>6.5</v>
+      </c>
+      <c r="K27">
+        <v>-6.5</v>
+      </c>
+      <c r="L27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="2">
+        <v>46206.49122685185</v>
+      </c>
+      <c r="G28">
+        <v>7.4145</v>
+      </c>
+      <c r="H28">
+        <v>-2.9358</v>
+      </c>
+      <c r="I28">
+        <v>1.056072807017544</v>
+      </c>
+      <c r="J28">
+        <v>6.5</v>
+      </c>
+      <c r="K28">
+        <v>-6.5</v>
+      </c>
+      <c r="L28" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
v3.1: feat - AOI_RS
</commit_message>
<xml_diff>
--- a/resources/M626/spc_sheet_oos_detail.xlsx
+++ b/resources/M626/spc_sheet_oos_detail.xlsx
@@ -679,7 +679,7 @@
         <v>-7.3274</v>
       </c>
       <c r="I5">
-        <v>0.02795575221238938</v>
+        <v>0.02795575221238939</v>
       </c>
       <c r="J5">
         <v>6.5</v>
@@ -869,7 +869,7 @@
         <v>-7.298</v>
       </c>
       <c r="I10">
-        <v>-0.8348867256637169</v>
+        <v>-0.8348867256637167</v>
       </c>
       <c r="J10">
         <v>6.5</v>
@@ -983,7 +983,7 @@
         <v>-4.1674</v>
       </c>
       <c r="I13">
-        <v>0.03299017857142859</v>
+        <v>0.0329901785714286</v>
       </c>
       <c r="J13">
         <v>6.5</v>
@@ -1439,7 +1439,7 @@
         <v>-3.8887</v>
       </c>
       <c r="I25">
-        <v>-0.09209473684210526</v>
+        <v>-0.09209473684210528</v>
       </c>
       <c r="J25">
         <v>6.5</v>
@@ -1477,7 +1477,7 @@
         <v>-5.5588</v>
       </c>
       <c r="I26">
-        <v>-0.97159203539823</v>
+        <v>-0.9715920353982301</v>
       </c>
       <c r="J26">
         <v>6.5</v>

</xml_diff>